<commit_message>
Fix EON June segment mapping
</commit_message>
<xml_diff>
--- a/estrazioni_tariffe/eon_tariffe_2026-06.xlsx
+++ b/estrazioni_tariffe/eon_tariffe_2026-06.xlsx
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+          <t>Quota fissa annua; per business include anche gestione energetica fissa.</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+          <t>Quota fissa annua; per business include anche gestione energetica fissa.</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+          <t>Quota fissa annua; per business include anche gestione energetica fissa.</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+          <t>Quota fissa annua; per business include anche gestione energetica fissa.</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MICROBUSINESS</t>
+          <t>BUSINESS</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">

</xml_diff>